<commit_message>
Data + Bar Chart done
</commit_message>
<xml_diff>
--- a/final-project/Final Info.xlsx
+++ b/final-project/Final Info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04e209669d46d7b2/Documents/College/Spring 2026/CSCI 344/final-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_F25DC773A252ABDACC1048AC699965185ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8990D27B-D13F-4796-A570-11327A067407}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="11_F25DC773A252ABDACC1048AC699965185ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B1277AF-69E1-40E9-B120-4690E3C033EF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -39,33 +39,15 @@
     <t>title</t>
   </si>
   <si>
-    <t>total sales</t>
-  </si>
-  <si>
-    <t>price</t>
-  </si>
-  <si>
     <t>photo</t>
   </si>
   <si>
-    <t>total copies sold</t>
-  </si>
-  <si>
-    <t>Monster Hunter</t>
-  </si>
-  <si>
     <t>Monster Hunter Freedom</t>
   </si>
   <si>
     <t>Monster Hunter Freedom 2</t>
   </si>
   <si>
-    <t>Monster Hunter Freedom Unite</t>
-  </si>
-  <si>
-    <t>Monster Hunter 3</t>
-  </si>
-  <si>
     <t>Monster Hunter 3 Ultimate</t>
   </si>
   <si>
@@ -78,13 +60,52 @@
     <t>Monster Hunter Generations Ultimate</t>
   </si>
   <si>
-    <t>Monster Hunter Rise/Sunbreak</t>
-  </si>
-  <si>
-    <t>Monster Hunter World/Iceborn</t>
+    <t>Monster Hunter World</t>
   </si>
   <si>
     <t>Monster Hunter Wilds</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/118170.png</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/16081.png</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/11009.png</t>
+  </si>
+  <si>
+    <t>Monster Hunter Rise</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/11019.png</t>
+  </si>
+  <si>
+    <t>Monster Hunter World: Iceborn</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/16149.png</t>
+  </si>
+  <si>
+    <t>Monster Hunter Rise: Sunbreak</t>
+  </si>
+  <si>
+    <t>https://cdn.promo.capcomusa.com/boxart/111061.png</t>
+  </si>
+  <si>
+    <t>total units sold (million)</t>
+  </si>
+  <si>
+    <t>Monster Hunter 4</t>
+  </si>
+  <si>
+    <t>Release Date</t>
+  </si>
+  <si>
+    <t>Monster Hunter Tri (3)</t>
+  </si>
+  <si>
+    <t>JP data</t>
   </si>
 </sst>
 </file>
@@ -123,9 +144,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,10 +430,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2">
+        <v>46022</v>
+      </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -422,113 +452,195 @@
       <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="1"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="F3" s="1"/>
+      <c r="G3" s="4">
+        <v>38687</v>
+      </c>
+      <c r="I3">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="F4" s="1"/>
+      <c r="G4" s="4">
+        <v>39114</v>
+      </c>
+      <c r="I4">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="4">
+        <v>40026</v>
+      </c>
+      <c r="I5">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E2" t="s">
+      <c r="F6" s="1"/>
+      <c r="G6" s="4">
+        <v>40878</v>
+      </c>
+      <c r="I6">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="4">
+        <v>41518</v>
+      </c>
+      <c r="I7">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E3" t="s">
+      <c r="F8" s="1"/>
+      <c r="G8" s="4">
+        <v>41913</v>
+      </c>
+      <c r="I8">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E4" t="s">
+      <c r="F9" s="1"/>
+      <c r="G9" s="4">
+        <v>42309</v>
+      </c>
+      <c r="I9">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E5" t="s">
+      <c r="F10" s="1"/>
+      <c r="G10" s="4">
+        <v>42795</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E6" t="s">
+      <c r="F11" s="1"/>
+      <c r="G11" s="4">
+        <v>43101</v>
+      </c>
+      <c r="H11" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="4">
+        <v>43709</v>
+      </c>
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12">
+        <v>15.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="4">
+        <v>44256</v>
+      </c>
+      <c r="H13" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13">
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="4">
+        <v>44713</v>
+      </c>
+      <c r="H14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I14">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E7" t="s">
+      <c r="F15" s="1"/>
+      <c r="G15" s="4">
+        <v>45689</v>
+      </c>
+      <c r="H15" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="E13" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0</v>
+      <c r="I15">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>